<commit_message>
Update negative price analysis 2026-03
</commit_message>
<xml_diff>
--- a/outputs/NSW_negative_prices.xlsx
+++ b/outputs/NSW_negative_prices.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Percentages" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Percentages" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Heatmap" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Audit" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Update pipeline outputs Apr 2026
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/NSW_negative_prices.xlsx
+++ b/outputs/NSW_negative_prices.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Percentages" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Heatmap" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Audit" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Percentages" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J83"/>
+  <dimension ref="A1:J84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3304,6 +3304,40 @@
         <v>0</v>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="n">
+        <v>13.51</v>
+      </c>
+      <c r="C84" s="3" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J84" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3315,7 +3349,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J83"/>
+  <dimension ref="A1:J84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6170,8 +6204,42 @@
         <v>0</v>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="n">
+        <v>13.51</v>
+      </c>
+      <c r="C84" s="3" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J84" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:B83">
+  <conditionalFormatting sqref="B2:B84">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -6183,7 +6251,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C83">
+  <conditionalFormatting sqref="C2:C84">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -6195,7 +6263,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D83">
+  <conditionalFormatting sqref="D2:D84">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -6207,7 +6275,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E83">
+  <conditionalFormatting sqref="E2:E84">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -6219,7 +6287,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F83">
+  <conditionalFormatting sqref="F2:F84">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -6231,7 +6299,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G83">
+  <conditionalFormatting sqref="G2:G84">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
@@ -6243,7 +6311,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H83">
+  <conditionalFormatting sqref="H2:H84">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
@@ -6255,7 +6323,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I83">
+  <conditionalFormatting sqref="I2:I84">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
@@ -6267,7 +6335,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J83">
+  <conditionalFormatting sqref="J2:J84">
     <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
@@ -6289,7 +6357,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K83"/>
+  <dimension ref="A1:K84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9396,6 +9464,43 @@
         <v>0</v>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" s="5" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="B84" s="5" t="n">
+        <v>2976</v>
+      </c>
+      <c r="C84" s="6" t="n">
+        <v>402</v>
+      </c>
+      <c r="D84" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E84" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F84" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I84" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J84" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K84" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>